<commit_message>
feat(ghfdb): complete 002 import/export pipeline and split specs
</commit_message>
<xml_diff>
--- a/tests/test_ghfdb/fixtures/sample_ghfdb.xlsx
+++ b/tests/test_ghfdb/fixtures/sample_ghfdb.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP10"/>
+  <dimension ref="A1:BP11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1138,172 +1138,342 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PARENT-001</t>
+          <t>allowed range: ID_parent</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>allowed range: q</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>allowed range: q_uncertainty</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Roundtrip Site</t>
+          <t>allowed range: name</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>allowed range: lat_NS</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>allowed range: long_EW</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>allowed range: elevation</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>onshore_continental</t>
+          <t>allowed range: environment</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>parent comment</t>
+          <t>allowed range: p_comment</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>allowed range: corr_HP_flag</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>allowed range: total_depth_MD</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>allowed range: total_depth_TVD</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>allowed range: explo_method</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Hydrocarbon</t>
+          <t>allowed range: explo_purpose</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>allowed range: Country</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Bavaria</t>
+          <t>allowed range: Region</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>allowed range: Continent</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>allowed range: Domain</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>CHILD-001</t>
+          <t>allowed range: ID</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>allowed range: qc</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>allowed range: qc_uncertainty</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Bullard method</t>
+          <t>allowed range: q_method</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>allowed range: q_top</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>allowed range: q_bottom</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>allowed range: probe_penetration</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>allowed range: publication_reference</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>allowed range: data_reference</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>allowed range: relevant_child</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>child-corrections</t>
+          <t>allowed range: c_comment</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>present_corrected</t>
+          <t>allowed range: corr_IS_flag</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>present_not_corrected</t>
+          <t>allowed range: corr_T_flag</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>present_not_significant</t>
+          <t>allowed range: corr_S_flag</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>not_recognized</t>
+          <t>allowed range: corr_E_flag</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>considered_p</t>
+          <t>allowed range: corr_TOPO_flag</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>considered_t</t>
+          <t>allowed range: corr_PAL_flag</t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>considered_pt</t>
+          <t>allowed range: corr_SUR_flag</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>not_considered</t>
+          <t>allowed range: corr_CONV_flag</t>
         </is>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>present_not_significant</t>
+          <t>allowed range: corr_HR_flag</t>
         </is>
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>Expedition A</t>
+          <t>allowed range: expedition</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>allowed range: probe_type</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>allowed range: probe_length</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>allowed range: probe_tilt</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>allowed range: water_temperature</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>allowed range: geo_lithology</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>allowed range: geo_stratigraphy</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>allowed range: T_grad_mean</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>allowed range: T_grad_uncertainty</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>allowed range: T_grad_mean_cor</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>allowed range: T_grad_uncertainty_cor</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>allowed range: T_method_top</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>allowed range: T_method_bottom</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>allowed range: T_shutin_top</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>allowed range: T_shutin_bottom</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>allowed range: T_corr_top</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>allowed range: T_corr_bottom</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>allowed range: T_number</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>allowed range: q_date</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_mean</t>
+        </is>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_uncertainty</t>
+        </is>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_source</t>
+        </is>
+      </c>
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_location</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_method</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_saturation</t>
+        </is>
+      </c>
+      <c r="BL8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_pT_conditions</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_pT_function</t>
+        </is>
+      </c>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_number</t>
+        </is>
+      </c>
+      <c r="BO8" t="inlineStr">
+        <is>
+          <t>allowed range: tc_strategy</t>
+        </is>
+      </c>
+      <c r="BP8" t="inlineStr">
+        <is>
+          <t>allowed range: igsn</t>
         </is>
       </c>
     </row>
@@ -1390,39 +1560,34 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>CHILD-002</t>
+          <t>CHILD-001</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>68</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Interval method</t>
+          <t>Bullard method</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
           <t>200</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB9" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1430,177 +1595,57 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>child-gradient-conductivity</t>
+          <t>child-corrections</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>present_corrected</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>present_not_corrected</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>present_not_significant</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>not_recognized</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>considered_p</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>considered_t</t>
         </is>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>considered_pt</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>not_considered</t>
         </is>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>present_not_significant</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
         <is>
-          <t>Expedition B</t>
-        </is>
-      </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AT9" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AU9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AV9" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="AW9" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="AX9" t="inlineStr">
-        <is>
-          <t>BHT</t>
-        </is>
-      </c>
-      <c r="AY9" t="inlineStr">
-        <is>
-          <t>BLK</t>
-        </is>
-      </c>
-      <c r="AZ9" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="BA9" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="BB9" t="inlineStr">
-        <is>
-          <t>AAPG correction</t>
-        </is>
-      </c>
-      <c r="BC9" t="inlineStr">
-        <is>
-          <t>Horner plot</t>
-        </is>
-      </c>
-      <c r="BD9" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="BF9" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="BG9" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="BH9" t="inlineStr">
-        <is>
-          <t>Core samples</t>
-        </is>
-      </c>
-      <c r="BI9" t="inlineStr">
-        <is>
-          <t>Actual heat-flow location</t>
-        </is>
-      </c>
-      <c r="BJ9" t="inlineStr">
-        <is>
-          <t>Estimation - from lithology and literature</t>
-        </is>
-      </c>
-      <c r="BK9" t="inlineStr">
-        <is>
-          <t>Dry measured</t>
-        </is>
-      </c>
-      <c r="BL9" t="inlineStr">
-        <is>
-          <t>Actual in-situ (pT) conditions</t>
-        </is>
-      </c>
-      <c r="BM9" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="BN9" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="BO9" t="inlineStr">
-        <is>
-          <t>Characterize formation conductivities</t>
+          <t>Expedition A</t>
         </is>
       </c>
     </row>
@@ -1687,85 +1732,382 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
+          <t>CHILD-002</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Interval method</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>child-gradient-conductivity</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>Expedition B</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>BHT</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>BLK</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>AAPG correction</t>
+        </is>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>Horner plot</t>
+        </is>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>Core samples</t>
+        </is>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>Actual heat-flow location</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>Estimation - from lithology and literature</t>
+        </is>
+      </c>
+      <c r="BK10" t="inlineStr">
+        <is>
+          <t>Dry measured</t>
+        </is>
+      </c>
+      <c r="BL10" t="inlineStr">
+        <is>
+          <t>Actual in-situ (pT) conditions</t>
+        </is>
+      </c>
+      <c r="BM10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="BN10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="BO10" t="inlineStr">
+        <is>
+          <t>Characterize formation conductivities</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PARENT-001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Roundtrip Site</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>onshore_continental</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>parent comment</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Hydrocarbon</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Bavaria</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
           <t>CHILD-003</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>Boot-strapping method</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>800</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AB11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>child-minimal</t>
         </is>
       </c>
-      <c r="AD10" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr">
+      <c r="AE11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF10" t="inlineStr">
+      <c r="AF11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AG10" t="inlineStr">
+      <c r="AG11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AH10" t="inlineStr">
+      <c r="AH11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AI10" t="inlineStr">
+      <c r="AI11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AJ10" t="inlineStr">
+      <c r="AJ11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AK10" t="inlineStr">
+      <c r="AK11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AL10" t="inlineStr">
+      <c r="AL11" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat(002-ghfdb-proxy): implement Phase 8 - replace local_id with ghfdb_id and add quality field
</commit_message>
<xml_diff>
--- a/tests/test_ghfdb/fixtures/sample_ghfdb.xlsx
+++ b/tests/test_ghfdb/fixtures/sample_ghfdb.xlsx
@@ -1478,10 +1478,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PARENT-001</t>
-        </is>
+      <c r="A9" t="n">
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1558,10 +1556,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>CHILD-001</t>
-        </is>
+      <c r="S9" t="n">
+        <v>1</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -1650,10 +1646,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>PARENT-001</t>
-        </is>
+      <c r="A10" t="n">
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1730,10 +1724,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>CHILD-002</t>
-        </is>
+      <c r="S10" t="n">
+        <v>2</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1947,10 +1939,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>PARENT-001</t>
-        </is>
+      <c r="A11" t="n">
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -2027,10 +2017,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>CHILD-003</t>
-        </is>
+      <c r="S11" t="n">
+        <v>3</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>

</xml_diff>